<commit_message>
replaced SJJ with SJW, removed oh4 and mdm
</commit_message>
<xml_diff>
--- a/continuous stations.xlsx
+++ b/continuous stations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawater-my.sharepoint.com/personal/rosemary_hartman_water_ca_gov/Documents/smelt cages/SMTWaterQuality/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="41" documentId="8_{72A71DD6-4F30-4CBC-B54E-21B51AEDE22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65ECA526-2A52-4A17-BE26-0AF894479B22}"/>
+  <xr:revisionPtr revIDLastSave="44" documentId="8_{72A71DD6-4F30-4CBC-B54E-21B51AEDE22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{26965903-DC6C-47AF-9BCA-710470476EA9}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{E43C89DB-75C2-428F-88E0-51B77BDDABCF}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{E43C89DB-75C2-428F-88E0-51B77BDDABCF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -69,9 +69,6 @@
     <t>OH4</t>
   </si>
   <si>
-    <t>SJJ</t>
-  </si>
-  <si>
     <t>WCI</t>
   </si>
   <si>
@@ -88,6 +85,9 @@
   </si>
   <si>
     <t>TWI</t>
+  </si>
+  <si>
+    <t>SJW</t>
   </si>
 </sst>
 </file>
@@ -97,7 +97,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,6 +116,12 @@
       <sz val="5"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF333333"/>
+      <name val="Source Sans Pro"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -145,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -158,6 +164,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -176,9 +183,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -216,7 +223,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -322,7 +329,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -464,7 +471,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -488,13 +495,13 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="4">
-        <v>38.052</v>
-      </c>
-      <c r="C2" s="5">
-        <v>-121.68899999999999</v>
+        <v>17</v>
+      </c>
+      <c r="B2" s="6">
+        <v>38.052002999999999</v>
+      </c>
+      <c r="C2" s="6">
+        <v>-121.689211</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -565,7 +572,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" s="4">
         <v>37.831600000000002</v>
@@ -598,7 +605,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="5">
         <v>37.963000000000001</v>
@@ -609,7 +616,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="5">
         <v>37.992800000000003</v>
@@ -620,7 +627,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="5">
         <v>38.066000000000003</v>
@@ -631,7 +638,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="5">
         <v>38.096400000000003</v>
@@ -642,7 +649,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="5">
         <v>38.096899999999998</v>

</xml_diff>